<commit_message>
feat(expenses): fatal parse-sanity gate before statement persist
Reject nonsense parses (bad dates/amounts, blank/mojibake merchants,
beyond-tolerance footer totals) with ParseSanityError so no statement or
tx rows are written; soft in-tolerance deltas and unmapped tx-types warn
only. Align max/isracard minimal fixtures so declared totals match.
</commit_message>
<xml_diff>
--- a/tests/fixtures/expenses/max_minimal.xlsx
+++ b/tests/fixtures/expenses/max_minimal.xlsx
@@ -536,10 +536,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-2097.83</v>
+        <v>-268.43</v>
       </c>
       <c r="D7" t="n">
-        <v>-2097.83</v>
+        <v>-268.43</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>

</xml_diff>